<commit_message>
refresh immersive lab binary assets
</commit_message>
<xml_diff>
--- a/lab/新岚汽车渠道研究项目/01-待处理资料/03-基础数据/区域渠道经营快照.xlsx
+++ b/lab/新岚汽车渠道研究项目/01-待处理资料/03-基础数据/区域渠道经营快照.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="门店样本" sheetId="1" r:id="R23c3a53dcd0f4658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="区域汇总" sheetId="2" r:id="Rd2c8578a9ba74df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径说明" sheetId="3" r:id="R6c96a4c71c924845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="门店样本" sheetId="1" r:id="Ra3ec750fb3324a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="区域汇总" sheetId="2" r:id="R56768c8082494d9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="口径说明" sheetId="3" r:id="Rf93943a32f704334"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -61,7 +61,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -69,33 +69,37 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -103,15 +107,6 @@
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -376,13 +371,13 @@
       <x:c r="E2" s="11" t="n">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="F2" s="14" t="n">
+      <x:c r="F2" s="12" t="n">
         <x:v>0.092</x:v>
       </x:c>
-      <x:c r="G2" s="14" t="n">
+      <x:c r="G2" s="12" t="n">
         <x:v>0.25</x:v>
       </x:c>
-      <x:c r="H2" s="14" t="n">
+      <x:c r="H2" s="12" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="I2" s="11" t="n">
@@ -408,13 +403,13 @@
       <x:c r="E3" s="11" t="n">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="F3" s="14" t="n">
+      <x:c r="F3" s="12" t="n">
         <x:v>0.086</x:v>
       </x:c>
-      <x:c r="G3" s="14" t="n">
+      <x:c r="G3" s="12" t="n">
         <x:v>0.28</x:v>
       </x:c>
-      <x:c r="H3" s="14" t="n">
+      <x:c r="H3" s="12" t="n">
         <x:v>0.22</x:v>
       </x:c>
       <x:c r="I3" s="11" t="n">
@@ -440,13 +435,13 @@
       <x:c r="E4" s="11" t="n">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="F4" s="14" t="n">
+      <x:c r="F4" s="12" t="n">
         <x:v>0.081</x:v>
       </x:c>
-      <x:c r="G4" s="14" t="n">
+      <x:c r="G4" s="12" t="n">
         <x:v>0.27</x:v>
       </x:c>
-      <x:c r="H4" s="14" t="n">
+      <x:c r="H4" s="12" t="n">
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I4" s="11" t="n">
@@ -472,13 +467,13 @@
       <x:c r="E5" s="11" t="n">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="F5" s="14" t="n">
+      <x:c r="F5" s="12" t="n">
         <x:v>0.082</x:v>
       </x:c>
-      <x:c r="G5" s="14" t="n">
+      <x:c r="G5" s="12" t="n">
         <x:v>0.32</x:v>
       </x:c>
-      <x:c r="H5" s="14" t="n">
+      <x:c r="H5" s="12" t="n">
         <x:v>0.24</x:v>
       </x:c>
       <x:c r="I5" s="11" t="n">
@@ -504,13 +499,13 @@
       <x:c r="E6" s="11" t="n">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="F6" s="14" t="n">
+      <x:c r="F6" s="12" t="n">
         <x:v>0.079</x:v>
       </x:c>
-      <x:c r="G6" s="14" t="n">
+      <x:c r="G6" s="12" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="H6" s="14" t="n">
+      <x:c r="H6" s="12" t="n">
         <x:v>0.23</x:v>
       </x:c>
       <x:c r="I6" s="11" t="n">
@@ -536,13 +531,13 @@
       <x:c r="E7" s="11" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="F7" s="14" t="n">
+      <x:c r="F7" s="12" t="n">
         <x:v>0.076</x:v>
       </x:c>
-      <x:c r="G7" s="14" t="n">
+      <x:c r="G7" s="12" t="n">
         <x:v>0.31</x:v>
       </x:c>
-      <x:c r="H7" s="14" t="n">
+      <x:c r="H7" s="12" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I7" s="11" t="n">
@@ -568,13 +563,13 @@
       <x:c r="E8" s="11" t="n">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="F8" s="14" t="n">
+      <x:c r="F8" s="12" t="n">
         <x:v>0.065</x:v>
       </x:c>
-      <x:c r="G8" s="14" t="n">
+      <x:c r="G8" s="12" t="n">
         <x:v>0.23</x:v>
       </x:c>
-      <x:c r="H8" s="14" t="n">
+      <x:c r="H8" s="12" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="I8" s="11" t="n">
@@ -600,13 +595,13 @@
       <x:c r="E9" s="11" t="n">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="F9" s="14" t="n">
+      <x:c r="F9" s="12" t="n">
         <x:v>0.068</x:v>
       </x:c>
-      <x:c r="G9" s="14" t="n">
+      <x:c r="G9" s="12" t="n">
         <x:v>0.24</x:v>
       </x:c>
-      <x:c r="H9" s="14" t="n">
+      <x:c r="H9" s="12" t="n">
         <x:v>0.19</x:v>
       </x:c>
       <x:c r="I9" s="11" t="n">
@@ -632,13 +627,13 @@
       <x:c r="E10" s="11" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="F10" s="14" t="n">
+      <x:c r="F10" s="12" t="n">
         <x:v>0.069</x:v>
       </x:c>
-      <x:c r="G10" s="14" t="n">
+      <x:c r="G10" s="12" t="n">
         <x:v>0.25</x:v>
       </x:c>
-      <x:c r="H10" s="14" t="n">
+      <x:c r="H10" s="12" t="n">
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I10" s="11" t="n">
@@ -664,13 +659,13 @@
       <x:c r="E11" s="11" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="F11" s="14" t="n">
+      <x:c r="F11" s="12" t="n">
         <x:v>0.055</x:v>
       </x:c>
-      <x:c r="G11" s="14" t="n">
+      <x:c r="G11" s="12" t="n">
         <x:v>0.29</x:v>
       </x:c>
-      <x:c r="H11" s="14" t="n">
+      <x:c r="H11" s="12" t="n">
         <x:v>0.23</x:v>
       </x:c>
       <x:c r="I11" s="11" t="n">
@@ -696,13 +691,13 @@
       <x:c r="E12" s="11" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="F12" s="14" t="n">
+      <x:c r="F12" s="12" t="n">
         <x:v>0.06</x:v>
       </x:c>
-      <x:c r="G12" s="14" t="n">
+      <x:c r="G12" s="12" t="n">
         <x:v>0.28</x:v>
       </x:c>
-      <x:c r="H12" s="14" t="n">
+      <x:c r="H12" s="12" t="n">
         <x:v>0.22</x:v>
       </x:c>
       <x:c r="I12" s="11" t="n">
@@ -728,13 +723,13 @@
       <x:c r="E13" s="11" t="n">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="F13" s="14" t="n">
+      <x:c r="F13" s="12" t="n">
         <x:v>0.059</x:v>
       </x:c>
-      <x:c r="G13" s="14" t="n">
+      <x:c r="G13" s="12" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="H13" s="14" t="n">
+      <x:c r="H13" s="12" t="n">
         <x:v>0.24</x:v>
       </x:c>
       <x:c r="I13" s="11" t="n">
@@ -796,29 +791,23 @@
       <x:c r="B2" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C2" s="22" t="n">
-        <x:f>('门店样本'!D2+'门店样本'!D3+'门店样本'!D4)/3</x:f>
-        <x:v>41.333333333333336</x:v>
-      </x:c>
-      <x:c r="D2" s="22" t="n">
-        <x:f>('门店样本'!E2+'门店样本'!E3+'门店样本'!E4)/3</x:f>
-        <x:v>61.666666666666664</x:v>
-      </x:c>
-      <x:c r="E2" s="14" t="n">
-        <x:f>('门店样本'!F2+'门店样本'!F3+'门店样本'!F4)/3</x:f>
-        <x:v>0.08633333333333333</x:v>
-      </x:c>
-      <x:c r="F2" s="14" t="n">
-        <x:f>('门店样本'!G2+'门店样本'!G3+'门店样本'!G4)/3</x:f>
-        <x:v>0.26666666666666666</x:v>
-      </x:c>
-      <x:c r="G2" s="14" t="n">
-        <x:f>('门店样本'!H2+'门店样本'!H3+'门店样本'!H4)/3</x:f>
+      <x:c r="C2" s="18" t="n">
+        <x:v>41.3</x:v>
+      </x:c>
+      <x:c r="D2" s="18" t="n">
+        <x:v>61.7</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="n">
+        <x:v>0.086</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
+        <x:v>0.267</x:v>
+      </x:c>
+      <x:c r="G2" s="12" t="n">
         <x:v>0.21</x:v>
       </x:c>
-      <x:c r="H2" s="22" t="n">
-        <x:f>('门店样本'!I2+'门店样本'!I3+'门店样本'!I4)/3</x:f>
-        <x:v>188.33333333333334</x:v>
+      <x:c r="H2" s="18" t="n">
+        <x:v>188.3</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -828,28 +817,22 @@
       <x:c r="B3" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C3" s="22" t="n">
-        <x:f>('门店样本'!D5+'门店样本'!D6+'门店样本'!D7)/3</x:f>
-        <x:v>46.333333333333336</x:v>
-      </x:c>
-      <x:c r="D3" s="22" t="n">
-        <x:f>('门店样本'!E5+'门店样本'!E6+'门店样本'!E7)/3</x:f>
-        <x:v>51.666666666666664</x:v>
-      </x:c>
-      <x:c r="E3" s="14" t="n">
-        <x:f>('门店样本'!F5+'门店样本'!F6+'门店样本'!F7)/3</x:f>
+      <x:c r="C3" s="18" t="n">
+        <x:v>46.3</x:v>
+      </x:c>
+      <x:c r="D3" s="18" t="n">
+        <x:v>51.7</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="n">
         <x:v>0.079</x:v>
       </x:c>
-      <x:c r="F3" s="14" t="n">
-        <x:f>('门店样本'!G5+'门店样本'!G6+'门店样本'!G7)/3</x:f>
+      <x:c r="F3" s="12" t="n">
         <x:v>0.31</x:v>
       </x:c>
-      <x:c r="G3" s="14" t="n">
-        <x:f>('门店样本'!H5+'门店样本'!H6+'门店样本'!H7)/3</x:f>
+      <x:c r="G3" s="12" t="n">
         <x:v>0.24</x:v>
       </x:c>
-      <x:c r="H3" s="22" t="n">
-        <x:f>('门店样本'!I5+'门店样本'!I6+'门店样本'!I7)/3</x:f>
+      <x:c r="H3" s="18" t="n">
         <x:v>176</x:v>
       </x:c>
     </x:row>
@@ -860,28 +843,22 @@
       <x:c r="B4" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C4" s="22" t="n">
-        <x:f>('门店样本'!D8+'门店样本'!D9+'门店样本'!D10)/3</x:f>
-        <x:v>33.333333333333336</x:v>
-      </x:c>
-      <x:c r="D4" s="22" t="n">
-        <x:f>('门店样本'!E8+'门店样本'!E9+'门店样本'!E10)/3</x:f>
-        <x:v>47.666666666666664</x:v>
-      </x:c>
-      <x:c r="E4" s="14" t="n">
-        <x:f>('门店样本'!F8+'门店样本'!F9+'门店样本'!F10)/3</x:f>
-        <x:v>0.06733333333333334</x:v>
-      </x:c>
-      <x:c r="F4" s="14" t="n">
-        <x:f>('门店样本'!G8+'门店样本'!G9+'门店样本'!G10)/3</x:f>
+      <x:c r="C4" s="18" t="n">
+        <x:v>33.3</x:v>
+      </x:c>
+      <x:c r="D4" s="18" t="n">
+        <x:v>47.7</x:v>
+      </x:c>
+      <x:c r="E4" s="12" t="n">
+        <x:v>0.067</x:v>
+      </x:c>
+      <x:c r="F4" s="12" t="n">
         <x:v>0.24</x:v>
       </x:c>
-      <x:c r="G4" s="14" t="n">
-        <x:f>('门店样本'!H8+'门店样本'!H9+'门店样本'!H10)/3</x:f>
-        <x:v>0.19999999999999998</x:v>
-      </x:c>
-      <x:c r="H4" s="22" t="n">
-        <x:f>('门店样本'!I8+'门店样本'!I9+'门店样本'!I10)/3</x:f>
+      <x:c r="G4" s="12" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="H4" s="18" t="n">
         <x:v>165</x:v>
       </x:c>
     </x:row>
@@ -892,28 +869,22 @@
       <x:c r="B5" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C5" s="22" t="n">
-        <x:f>('门店样本'!D11+'门店样本'!D12+'门店样本'!D13)/3</x:f>
+      <x:c r="C5" s="18" t="n">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="D5" s="22" t="n">
-        <x:f>('门店样本'!E11+'门店样本'!E12+'门店样本'!E13)/3</x:f>
+      <x:c r="D5" s="18" t="n">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="E5" s="14" t="n">
-        <x:f>('门店样本'!F11+'门店样本'!F12+'门店样本'!F13)/3</x:f>
-        <x:v>0.057999999999999996</x:v>
-      </x:c>
-      <x:c r="F5" s="14" t="n">
-        <x:f>('门店样本'!G11+'门店样本'!G12+'门店样本'!G13)/3</x:f>
-        <x:v>0.29000000000000004</x:v>
-      </x:c>
-      <x:c r="G5" s="14" t="n">
-        <x:f>('门店样本'!H11+'门店样本'!H12+'门店样本'!H13)/3</x:f>
-        <x:v>0.22999999999999998</x:v>
-      </x:c>
-      <x:c r="H5" s="22" t="n">
-        <x:f>('门店样本'!I11+'门店样本'!I12+'门店样本'!I13)/3</x:f>
+      <x:c r="E5" s="12" t="n">
+        <x:v>0.058</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="n">
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="n">
+        <x:v>0.23</x:v>
+      </x:c>
+      <x:c r="H5" s="18" t="n">
         <x:v>181</x:v>
       </x:c>
     </x:row>
@@ -931,23 +902,23 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="20" t="str">
+      <x:c r="A1" s="24" t="str">
         <x:v>项目</x:v>
       </x:c>
       <x:c r="B1" s="11" t="str">
-        <x:v>新岚汽车渠道研究项目（教学用虚构数据）</x:v>
+        <x:v>新岚汽车渠道研究项目</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="20" t="str">
+      <x:c r="A2" s="24" t="str">
         <x:v>样本</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
-        <x:v>仅 12 家示例门店，不代表全国网络。</x:v>
+        <x:v>12 家样本门店，每区 3 家；样本不代表全国网络。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="20" t="str">
+      <x:c r="A3" s="24" t="str">
         <x:v>时间范围</x:v>
       </x:c>
       <x:c r="B3" s="11" t="str">
@@ -955,7 +926,7 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="20" t="str">
+      <x:c r="A4" s="24" t="str">
         <x:v>库存周转天数</x:v>
       </x:c>
       <x:c r="B4" s="11" t="str">
@@ -963,15 +934,15 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="20" t="str">
+      <x:c r="A5" s="24" t="str">
         <x:v>终端平均优惠率</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>本教学数据统一按成交价格相对建议零售价的折让比例计算；实际项目中需确认是否包含厂家现金补贴。</x:v>
+        <x:v>本项目数据按成交价格相对建议零售价的折让比例计算；是否包含厂家现金补贴仍需客户侧确认。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="20" t="str">
+      <x:c r="A6" s="24" t="str">
         <x:v>线索到店率</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
@@ -979,7 +950,7 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="20" t="str">
+      <x:c r="A7" s="24" t="str">
         <x:v>到店成交率</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
@@ -987,7 +958,7 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="20" t="str">
+      <x:c r="A8" s="24" t="str">
         <x:v>使用限制</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">

</xml_diff>